<commit_message>
data processing basics, docu for relevant cols
</commit_message>
<xml_diff>
--- a/relevant_cols.xlsx
+++ b/relevant_cols.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonas\Documents\GitHub\datathon_make_it_strong\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{175ABCB7-665B-4882-9D22-50784C00C09A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E7B60A6-5788-4FDC-A074-19671AF4F1D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8F3E04FF-84EE-472A-A48A-CE946EAA8C48}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>name</t>
   </si>
@@ -110,24 +110,6 @@
     <t>wave 3 weights</t>
   </si>
   <si>
-    <t>w3sq61</t>
-  </si>
-  <si>
-    <t>Would face negative work-related consequences after parenta leave in [country]</t>
-  </si>
-  <si>
-    <t>w4sq2</t>
-  </si>
-  <si>
-    <t>Importance of family in life</t>
-  </si>
-  <si>
-    <t>w4sq11</t>
-  </si>
-  <si>
-    <t>Importance of children in a marriage/partnerhsip</t>
-  </si>
-  <si>
     <t>w5pspwght</t>
   </si>
   <si>
@@ -146,34 +128,37 @@
     <t>wave 4 weights</t>
   </si>
   <si>
-    <t>w5sq13</t>
-  </si>
-  <si>
-    <t>Financial ability to afford a/another child in next three years</t>
-  </si>
-  <si>
-    <t>w5sq14</t>
-  </si>
-  <si>
-    <t>Access to suitable housing for a/another child in next three years</t>
-  </si>
-  <si>
-    <t>Access to satisfactory childcare for a/another child in next three years</t>
-  </si>
-  <si>
-    <t>w5sq15</t>
-  </si>
-  <si>
-    <t>Access to sufficient paid parental leave for a/another child in next three years</t>
-  </si>
-  <si>
-    <t>w5sq16</t>
-  </si>
-  <si>
-    <t>Social policies where government should spend more money: Family policies</t>
-  </si>
-  <si>
-    <t>w5sq17_1</t>
+    <t>wave 2 weights</t>
+  </si>
+  <si>
+    <t>w3pspwght</t>
+  </si>
+  <si>
+    <t>w1sq3</t>
+  </si>
+  <si>
+    <t>w1sq2</t>
+  </si>
+  <si>
+    <t>Everyone in country fair chance achieve level of education they seek</t>
+  </si>
+  <si>
+    <t>w1sq1</t>
+  </si>
+  <si>
+    <t>Compared other people in country, fair chance achieve level of education I seek</t>
+  </si>
+  <si>
+    <t>Satisfaction with level of education you have reached</t>
+  </si>
+  <si>
+    <t>Correspondence between job and educational qualification</t>
+  </si>
+  <si>
+    <t>w3sq74</t>
+  </si>
+  <si>
+    <t xml:space="preserve">age </t>
   </si>
 </sst>
 </file>
@@ -228,13 +213,9 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C67AF9B-1123-477B-B3AA-C95E4C6FCAE6}" name="Tabelle1" displayName="Tabelle1" ref="A1:C23" totalsRowShown="0">
-  <autoFilter ref="A1:C23" xr:uid="{3C67AF9B-1123-477B-B3AA-C95E4C6FCAE6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3C67AF9B-1123-477B-B3AA-C95E4C6FCAE6}" name="Tabelle1" displayName="Tabelle1" ref="A1:C24" totalsRowShown="0">
+  <autoFilter ref="A1:C24" xr:uid="{3C67AF9B-1123-477B-B3AA-C95E4C6FCAE6}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{C720B57B-71A2-477C-8A4C-5E5D8BF01A03}" name="name"/>
     <tableColumn id="2" xr3:uid="{E4D8CFE9-98D6-4CD5-B1EA-43B5F265840D}" name="description"/>
@@ -561,7 +542,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{801FF945-DD69-418B-ABC7-9EBFC62F2E2B}">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="62.33203125" customWidth="1"/>
@@ -598,6 +579,9 @@
       <c r="A4" t="s">
         <v>7</v>
       </c>
+      <c r="B4" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
@@ -657,7 +641,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B12" t="s">
         <v>22</v>
@@ -668,21 +652,21 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B13" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C13">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C14">
         <v>3</v>
@@ -690,10 +674,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B15" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C15">
         <v>4</v>
@@ -701,90 +685,57 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B16" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C16">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="B17" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C17">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="B18" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C18">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B19" t="s">
         <v>37</v>
       </c>
       <c r="C19">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" t="s">
         <v>38</v>
       </c>
-      <c r="B20" t="s">
-        <v>39</v>
-      </c>
       <c r="C20">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
-        <v>41</v>
-      </c>
-      <c r="B21" t="s">
-        <v>40</v>
-      </c>
-      <c r="C21">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>43</v>
-      </c>
-      <c r="B22" t="s">
-        <v>42</v>
-      </c>
-      <c r="C22">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>45</v>
-      </c>
-      <c r="B23" t="s">
-        <v>44</v>
-      </c>
-      <c r="C23">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
preprocessing and relevant cols updated
</commit_message>
<xml_diff>
--- a/relevant_cols.xlsx
+++ b/relevant_cols.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonas\Documents\GitHub\datathon_make_it_strong\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86199ED3-6D7B-4567-92E8-70BDB40A66EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CF388F0-082D-4D53-ACC8-5FC7F9DB1D3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8F3E04FF-84EE-472A-A48A-CE946EAA8C48}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>name</t>
   </si>
@@ -159,6 +159,18 @@
   </si>
   <si>
     <t xml:space="preserve">age </t>
+  </si>
+  <si>
+    <t>w5hq5</t>
+  </si>
+  <si>
+    <t>Felt safe with at least one carer during first 18 years of life</t>
+  </si>
+  <si>
+    <t>w5hq8</t>
+  </si>
+  <si>
+    <t>Severe financial difficulties in family during first 18 years of life, how often</t>
   </si>
 </sst>
 </file>
@@ -542,7 +554,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{801FF945-DD69-418B-ABC7-9EBFC62F2E2B}">
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="62.33203125" customWidth="1"/>
@@ -738,10 +750,33 @@
         <v>3</v>
       </c>
     </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>41</v>
+      </c>
+      <c r="B21" t="s">
+        <v>42</v>
+      </c>
+      <c r="C21">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>